<commit_message>
Database testing and soft assertion code added
</commit_message>
<xml_diff>
--- a/src/test/resources/testData/TestData.xlsx
+++ b/src/test/resources/testData/TestData.xlsx
@@ -1,16 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29721"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29819"/>
   <workbookPr/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{4E1670E7-40E1-4F08-8C69-F7D8C6693600}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{2BE97D89-DEA9-4B87-848F-6622D87E8570}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="6800" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="6800" firstSheet="1" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="validLoginData" sheetId="1" r:id="rId1"/>
-    <sheet name="emplVerification" sheetId="3" r:id="rId2"/>
-    <sheet name="inValidLoginData" sheetId="2" r:id="rId3"/>
+    <sheet name="pim" sheetId="4" r:id="rId2"/>
+    <sheet name="emplVerification" sheetId="3" r:id="rId3"/>
+    <sheet name="inValidLoginData" sheetId="2" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191028"/>
   <extLst>
@@ -33,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="25">
   <si>
     <t>username</t>
   </si>
@@ -41,15 +42,18 @@
     <t>password</t>
   </si>
   <si>
-    <t>admin</t>
-  </si>
-  <si>
-    <t>admin123</t>
+    <t>hmahesh</t>
+  </si>
+  <si>
+    <t>Sanju@3124</t>
   </si>
   <si>
     <t>fname</t>
   </si>
   <si>
+    <t>mname</t>
+  </si>
+  <si>
     <t>lname</t>
   </si>
   <si>
@@ -59,7 +63,10 @@
     <t>MANGESH</t>
   </si>
   <si>
-    <t>KARANDE</t>
+    <t>SADANAND</t>
+  </si>
+  <si>
+    <t>YADAV</t>
   </si>
   <si>
     <t>0001</t>
@@ -68,6 +75,9 @@
     <t>SATISH</t>
   </si>
   <si>
+    <t>LALA</t>
+  </si>
+  <si>
     <t>JADHAV</t>
   </si>
   <si>
@@ -77,10 +87,22 @@
     <t>KALPESH</t>
   </si>
   <si>
+    <t>MAMA</t>
+  </si>
+  <si>
     <t>KALE</t>
   </si>
   <si>
     <t>0003</t>
+  </si>
+  <si>
+    <t>emp_id</t>
+  </si>
+  <si>
+    <t>emp_name</t>
+  </si>
+  <si>
+    <t>Hitendra</t>
   </si>
   <si>
     <t>admin1</t>
@@ -93,7 +115,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3">
+  <fonts count="4">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -112,6 +134,12 @@
       <color rgb="FF000000"/>
       <name val="Calibri"/>
       <charset val="1"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
     </font>
   </fonts>
   <fills count="2">
@@ -134,11 +162,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -414,8 +445,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B3"/>
+  <dimension ref="A1:B2"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.45"/>
+  <cols>
+    <col min="2" max="2" width="10.375" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" t="s">
@@ -433,66 +467,97 @@
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:2">
-      <c r="A3" t="s">
-        <v>2</v>
-      </c>
-      <c r="B3" t="s">
-        <v>3</v>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7B19EE2E-DCC8-483B-9012-403B44059F1C}">
-  <dimension ref="A1:C4"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{39DD9851-0A3A-4003-B1F2-21D935973F64}">
+  <dimension ref="A1:F4"/>
   <sheetFormatPr defaultRowHeight="13.5"/>
+  <cols>
+    <col min="4" max="4" width="9.625" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="14.25">
-      <c r="A1" t="s">
+    <row r="1" spans="1:6" ht="14.25">
+      <c r="A1" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
         <v>4</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="D1" t="s">
         <v>5</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="2" spans="1:3">
-      <c r="A2" t="s">
+      <c r="F1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="B2" t="s">
+    </row>
+    <row r="2" spans="1:6">
+      <c r="A2" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="C2" t="s">
         <v>8</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="D2" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="3" spans="1:3" ht="15">
-      <c r="A3" t="s">
+      <c r="E2" t="s">
         <v>10</v>
       </c>
-      <c r="B3" t="s">
+      <c r="F2" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="C3" s="3" t="s">
+    </row>
+    <row r="3" spans="1:6" ht="15">
+      <c r="A3" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="C3" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="4" spans="1:3">
-      <c r="A4" t="s">
+      <c r="D3" t="s">
         <v>13</v>
       </c>
-      <c r="B4" t="s">
+      <c r="E3" t="s">
         <v>14</v>
       </c>
-      <c r="C4" s="2" t="s">
+      <c r="F3" s="3" t="s">
         <v>15</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6">
+      <c r="A4" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="C4" t="s">
+        <v>16</v>
+      </c>
+      <c r="D4" t="s">
+        <v>17</v>
+      </c>
+      <c r="E4" t="s">
+        <v>18</v>
+      </c>
+      <c r="F4" s="2" t="s">
+        <v>19</v>
       </c>
     </row>
   </sheetData>
@@ -501,6 +566,49 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7B19EE2E-DCC8-483B-9012-403B44059F1C}">
+  <dimension ref="A1:F4"/>
+  <sheetFormatPr defaultRowHeight="13.5"/>
+  <cols>
+    <col min="2" max="2" width="9.375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="9.625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" ht="14.25">
+      <c r="A1" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="B1" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="E1" s="1"/>
+      <c r="F1" s="1"/>
+    </row>
+    <row r="2" spans="1:6">
+      <c r="A2" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="B2" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="F2" s="2"/>
+    </row>
+    <row r="3" spans="1:6" ht="15">
+      <c r="A3" s="4"/>
+      <c r="B3" s="4"/>
+      <c r="F3" s="3"/>
+    </row>
+    <row r="4" spans="1:6">
+      <c r="A4" s="4"/>
+      <c r="B4" s="4"/>
+      <c r="F4" s="2"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:B2"/>
   <sheetFormatPr defaultColWidth="8.75" defaultRowHeight="14.45"/>
@@ -515,10 +623,10 @@
     </row>
     <row r="2" spans="1:2">
       <c r="A2" t="s">
-        <v>16</v>
+        <v>23</v>
       </c>
       <c r="B2" t="s">
-        <v>17</v>
+        <v>24</v>
       </c>
     </row>
   </sheetData>

</xml_diff>